<commit_message>
Auto update Pengadaan 2026-08-20 15:36:28
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-20).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-08-20).xlsx
@@ -743,28 +743,28 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>381815300</v>
+        <v>317493140</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>51900000</v>
+        <v>19500000</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>51900000</v>
+        <v>19500000</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>329915300</v>
+        <v>297993140</v>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
@@ -961,22 +961,22 @@
         <v>491911485</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>84907554</v>
+        <v>84108354</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>78869208</v>
+        <v>78149208</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>407003931</v>
+        <v>407803131</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
@@ -1063,22 +1063,22 @@
         <v>908204422</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>322688209</v>
+        <v>278259519</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>302852413</v>
+        <v>258444643</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>585516213</v>
+        <v>629944903</v>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -1131,22 +1131,22 @@
         <v>2090003236</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1136240668</v>
+        <v>1116124360</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1115612710.6</v>
+        <v>1095681550.6</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>953762568</v>
+        <v>973878876</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -1165,22 +1165,22 @@
         <v>444206345</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>79101092</v>
+        <v>32101092</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>75945607</v>
+        <v>29240607</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>365105253</v>
+        <v>412105253</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -1199,22 +1199,22 @@
         <v>342136823</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>30262050</v>
+        <v>2661900</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>26778260</v>
+        <v>2476475</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>311874773</v>
+        <v>339474923</v>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
@@ -1227,22 +1227,22 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>794109241</v>
+        <v>775509241</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>99927566</v>
+        <v>81327566</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>94276500</v>
+        <v>75876500</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>116</v>
@@ -1295,28 +1295,28 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>2181596820</v>
+        <v>2238310494</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>319575637</v>
+        <v>275059798</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>316486817</v>
+        <v>272586367</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>1862021183</v>
+        <v>1963250696</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
@@ -1499,28 +1499,28 @@
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>880998213</v>
+        <v>867585528</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>580813055</v>
+        <v>518182970</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>494176948</v>
+        <v>440947598</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>300185158</v>
+        <v>349402558</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -1573,22 +1573,22 @@
         <v>550936395</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>73983300</v>
+        <v>20208300</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>73788167</v>
+        <v>20013167</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>476953095</v>
+        <v>530728095</v>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
@@ -1601,28 +1601,28 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>489056792</v>
+        <v>476139500</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>34949904</v>
+        <v>12917292</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>21152715</v>
+        <v>11908080</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>454106888</v>
+        <v>463222208</v>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
@@ -1641,22 +1641,22 @@
         <v>251691298</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>141795000</v>
+        <v>60000000</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>64745634</v>
+        <v>21674415</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>109896298</v>
+        <v>191691298</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -2115,10 +2115,10 @@
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>181249887</v>
+        <v>162372837</v>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
@@ -2141,10 +2141,10 @@
         </is>
       </c>
       <c r="I48" s="8" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="J48" s="10" t="n">
-        <v>181249887</v>
+        <v>162372837</v>
       </c>
     </row>
     <row r="49" ht="45" customHeight="1">
@@ -2653,10 +2653,10 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>164340083</v>
+        <v>193865001</v>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
@@ -2679,10 +2679,10 @@
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>164340083</v>
+        <v>193865001</v>
       </c>
     </row>
     <row r="62" ht="45" customHeight="1">
@@ -2777,22 +2777,22 @@
         <v>354293991</v>
       </c>
       <c r="E64" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>129198291</v>
+        <v>119763291</v>
       </c>
       <c r="G64" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H64" s="10" t="n">
-        <v>127533150</v>
+        <v>118233150</v>
       </c>
       <c r="I64" s="8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J64" s="10" t="n">
-        <v>225095700</v>
+        <v>234530700</v>
       </c>
     </row>
     <row r="65" ht="45" customHeight="1">
@@ -2871,28 +2871,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>3891</v>
+        <v>3879</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>32315561122</v>
+        <v>32273670527</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>375</v>
+        <v>349</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>6143937440</v>
+        <v>5678809556</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>375</v>
+        <v>349</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>5698927658.6</v>
+        <v>5299541289.6</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>3516</v>
+        <v>3530</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>26171623682</v>
+        <v>26594860971</v>
       </c>
     </row>
   </sheetData>
@@ -3259,41 +3259,41 @@
         <v>5</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>448925330</v>
+        <v>513247490</v>
       </c>
       <c r="E10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>190310330</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>173267420</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>173267420</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="10" t="n">
-        <v>276710330</v>
-      </c>
-      <c r="G10" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" s="10" t="n">
-        <v>259667420</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>259667420</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="8" t="n">
-        <v>2</v>
-      </c>
       <c r="N10" s="10" t="n">
-        <v>172215000</v>
+        <v>322937160</v>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
@@ -3624,22 +3624,22 @@
         <v>1566751699</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>1225542538</v>
+        <v>1095357742</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>896262562</v>
+        <v>767102962</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>896262562</v>
+        <v>767102962</v>
       </c>
       <c r="K17" s="4" t="n">
         <v>3</v>
@@ -3648,10 +3648,10 @@
         <v>237557765</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>341209161</v>
+        <v>471393957</v>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
@@ -3716,16 +3716,16 @@
         <v>1888168641</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1162285000</v>
+        <v>905090000</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1157390640</v>
+        <v>900653190</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>6</v>
@@ -3740,10 +3740,10 @@
         <v>194832750</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>725883641</v>
+        <v>983078641</v>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -3806,10 +3806,10 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>19564340479</v>
+        <v>19684340479</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>122</v>
@@ -3824,10 +3824,10 @@
         <v>16613057107.4</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>12101060134</v>
+        <v>11952908434</v>
       </c>
       <c r="K21" s="4" t="n">
         <v>1</v>
@@ -3836,10 +3836,10 @@
         <v>72965295</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2347995701</v>
+        <v>2467995701</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -4056,28 +4056,28 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>6465227440</v>
+        <v>6408513766</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>3847498984</v>
+        <v>2977701197</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>3821561702</v>
+        <v>2962395450</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>347319002</v>
+        <v>296952750</v>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -4090,10 +4090,10 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>2617728456</v>
+        <v>3430812569</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
@@ -4162,22 +4162,22 @@
         <v>5044708697</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>3591835307</v>
+        <v>3222242603</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>3578130623</v>
+        <v>3209499623</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J28" s="10" t="n">
-        <v>3065893618</v>
+        <v>2697262618</v>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="N28" s="10" t="n">
-        <v>1452873390</v>
+        <v>1822466094</v>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1">
@@ -4212,22 +4212,22 @@
         <v>2784104510</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>1179232601</v>
+        <v>743457601</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>1151500223</v>
+        <v>719438273</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>757394273</v>
+        <v>424838273</v>
       </c>
       <c r="K29" s="4" t="n">
         <v>1</v>
@@ -4236,10 +4236,10 @@
         <v>50500763</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>1604871909</v>
+        <v>2040646909</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -4366,22 +4366,22 @@
         <v>24100076698</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>23567530878</v>
+        <v>17335125078</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>23497213425.01</v>
+        <v>17280318880</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>2833129460</v>
+        <v>318354660</v>
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
@@ -4394,10 +4394,10 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="N32" s="10" t="n">
-        <v>532545820</v>
+        <v>6764951620</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -4602,22 +4602,22 @@
         <v>523391100</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>273952950</v>
+        <v>221982350</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>153319438</v>
+        <v>150899438</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>153319438</v>
+        <v>150899438</v>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
@@ -4630,10 +4630,10 @@
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N36" s="10" t="n">
-        <v>249438150</v>
+        <v>301408750</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -4825,23 +4825,35 @@
       <c r="D40" s="10" t="n">
         <v>320725524</v>
       </c>
-      <c r="E40" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="10" t="n">
-        <v>81320000</v>
-      </c>
-      <c r="G40" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="10" t="n">
-        <v>80619300</v>
-      </c>
-      <c r="I40" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J40" s="10" t="n">
-        <v>80619300</v>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K40" s="11" t="inlineStr">
         <is>
@@ -4854,10 +4866,10 @@
         </is>
       </c>
       <c r="M40" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N40" s="10" t="n">
-        <v>239405524</v>
+        <v>320725524</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -4990,28 +5002,28 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" s="6" t="n">
-        <v>403460838</v>
+        <v>302731124</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>340582172</v>
+        <v>239852458</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>68020787</v>
+        <v>65401200</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>68020787</v>
+        <v>65401200</v>
       </c>
       <c r="K43" s="7" t="inlineStr">
         <is>
@@ -5288,10 +5300,10 @@
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>145950000</v>
+        <v>50400000</v>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
@@ -5334,10 +5346,10 @@
         </is>
       </c>
       <c r="M48" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N48" s="10" t="n">
-        <v>145950000</v>
+        <v>50400000</v>
       </c>
     </row>
     <row r="49" ht="45" customHeight="1">
@@ -6265,17 +6277,25 @@
       <c r="D64" s="10" t="n">
         <v>463002876</v>
       </c>
-      <c r="E64" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F64" s="10" t="n">
-        <v>205350000</v>
-      </c>
-      <c r="G64" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H64" s="10" t="n">
-        <v>204500000</v>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
@@ -6298,10 +6318,10 @@
         </is>
       </c>
       <c r="M64" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N64" s="10" t="n">
-        <v>257652876</v>
+        <v>463002876</v>
       </c>
     </row>
     <row r="65" ht="45" customHeight="1">
@@ -6412,28 +6432,28 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>94843509132</v>
+        <v>94774837904</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>486</v>
+        <v>417</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>62300686991</v>
+        <v>53479965590</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>486</v>
+        <v>417</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>60375849277.41</v>
+        <v>51736639593.4</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>234</v>
+        <v>200</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>27927647334</v>
+        <v>24211949095</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>9</v>
@@ -6442,10 +6462,10 @@
         <v>764123653</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>314</v>
+        <v>381</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>32542822141</v>
+        <v>41294872314</v>
       </c>
     </row>
   </sheetData>
@@ -7250,19 +7270,19 @@
         <v>32</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>5375504750</v>
+        <v>3557204750</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>5375504750</v>
+        <v>3557204750</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>1987132203</v>
+        <v>1101458974</v>
       </c>
       <c r="M17" s="4" t="n">
         <v>2</v>
@@ -7461,22 +7481,22 @@
         <v>35948239265</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>33663796833</v>
+        <v>33346991733</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>32168354970</v>
+        <v>31855864970</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>31161310970</v>
+        <v>30848820970</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -7489,10 +7509,10 @@
         </is>
       </c>
       <c r="M21" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2284442432</v>
+        <v>2601247532</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -7620,25 +7640,37 @@
         <v>2</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>777000000</v>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>465000000</v>
-      </c>
-      <c r="G24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="10" t="n">
-        <v>462500000</v>
-      </c>
-      <c r="I24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>462500000</v>
+        <v>795600000</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
@@ -7651,10 +7683,10 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N24" s="10" t="n">
-        <v>312000000</v>
+        <v>795600000</v>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
@@ -7835,38 +7867,38 @@
         <v>2208956507</v>
       </c>
       <c r="E28" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>1062414494</v>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="10" t="n">
+        <v>1054476790</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>711476790</v>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F28" s="10" t="n">
-        <v>1280399846</v>
-      </c>
-      <c r="G28" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H28" s="10" t="n">
-        <v>1272380890</v>
-      </c>
-      <c r="I28" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="J28" s="10" t="n">
-        <v>929380890</v>
-      </c>
-      <c r="K28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L28" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M28" s="8" t="n">
-        <v>4</v>
-      </c>
       <c r="N28" s="10" t="n">
-        <v>928556661</v>
+        <v>1146542013</v>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1">
@@ -8001,22 +8033,22 @@
         <v>3813601480</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>3013841480</v>
+        <v>2375841480</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>2296738818</v>
+        <v>1661608818</v>
       </c>
       <c r="I31" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>2296738818</v>
+        <v>1661608818</v>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
@@ -8029,10 +8061,10 @@
         </is>
       </c>
       <c r="M31" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>799760000</v>
+        <v>1437760000</v>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
@@ -8048,19 +8080,19 @@
         <v>11</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>4274621970</v>
+        <v>3639664785</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>3786710370</v>
+        <v>545702400</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>2513539864.01</v>
+        <v>544900064</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>1</v>
@@ -8079,10 +8111,10 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="N32" s="10" t="n">
-        <v>487911600</v>
+        <v>3093962385</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -8269,28 +8301,28 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>15104060325</v>
+        <v>6878905700</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>11747602475</v>
+        <v>3522447850</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>293606685</v>
+        <v>173537400</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>293606685</v>
+        <v>173537400</v>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
@@ -10197,22 +10229,22 @@
         <v>5031291001</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>2470791364</v>
+        <v>218268000</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>1559826000</v>
+        <v>185076000</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>1559826000</v>
+        <v>185076000</v>
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
@@ -10225,10 +10257,10 @@
         </is>
       </c>
       <c r="M65" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N65" s="6" t="n">
-        <v>2560499637</v>
+        <v>4813023001</v>
       </c>
     </row>
     <row r="66" ht="45" customHeight="1">
@@ -10289,40 +10321,40 @@
         </is>
       </c>
       <c r="C67" s="12" t="n">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>170243233838</v>
+        <v>161401722028</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="F67" s="13" t="n">
-        <v>130114856886</v>
+        <v>114758380475</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>64077082121.01</v>
+        <v>57167298936</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>60018148321</v>
+        <v>55077004936</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="L67" s="13" t="n">
-        <v>2980144727</v>
+        <v>2094471498</v>
       </c>
       <c r="M67" s="12" t="n">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="N67" s="13" t="n">
-        <v>40128376952</v>
+        <v>46643341553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>